<commit_message>
ajuste para transportes ape, verificar ojo
</commit_message>
<xml_diff>
--- a/ejemplo_transporte.xlsx
+++ b/ejemplo_transporte.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t xml:space="preserve">NOMBRE PROFESIONAL</t>
   </si>
@@ -55,30 +55,32 @@
     <t xml:space="preserve">VALOR</t>
   </si>
   <si>
-    <t xml:space="preserve">ELIANA INES HERNANDEZ RODRIGUEZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANGELA MARILUZ GALLEGO </t>
+    <t xml:space="preserve">MIRIAN perez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIRIAN PEREZ</t>
   </si>
   <si>
     <t xml:space="preserve">d</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSPORTE NNA GUADALUPE GALLEGO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GLORIA MILENA CARMONA GIRALDO</t>
+    <t xml:space="preserve">TRANSPORTE APOYO A LA INCLUSION MES DE SEPTIEMBRE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRANSPORTENNAJACOBOBEDOYA QUINTERO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$100.000</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -124,21 +126,8 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -161,12 +150,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
         <bgColor rgb="FF003366"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -218,7 +201,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -243,32 +226,8 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -348,12 +307,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:K1048576"/>
+  <sheetFormatPr defaultColWidth="12.71484375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="47.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="25.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="33.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="29.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="41.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="66.83"/>
@@ -394,75 +354,43 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="7" t="n">
-        <v>1054546418</v>
-      </c>
-      <c r="C2" s="7" t="n">
-        <v>13809501</v>
-      </c>
-      <c r="D2" s="8" t="s">
+      <c r="B2" s="6" t="n">
+        <v>1054876999</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>23809501</v>
+      </c>
+      <c r="D2" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="8" t="n">
-        <v>42018286</v>
-      </c>
-      <c r="F2" s="8" t="s">
+      <c r="E2" s="6" t="n">
+        <v>1054876999</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="9" t="n">
-        <v>6165950521</v>
-      </c>
-      <c r="H2" s="7" t="s">
+      <c r="G2" s="6" t="n">
+        <v>6165950222</v>
+      </c>
+      <c r="H2" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" s="9" t="n">
-        <v>114</v>
-      </c>
-      <c r="K2" s="11" t="n">
-        <v>15000</v>
+      <c r="I2" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="0" t="n">
+        <v>113</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="8" t="n">
-        <v>24828302</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="12" t="n">
-        <v>6165950523</v>
-      </c>
-      <c r="H3" s="7"/>
-      <c r="I3" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="J3" s="9" t="n">
-        <v>114</v>
-      </c>
-      <c r="K3" s="11" t="n">
-        <v>15000</v>
-      </c>
-    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="H2:H3"/>
-  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>